<commit_message>
Portal: the inventory becomes Home — first tab, and where the site opens
Opening the portal landed on Provision, a form, rather than on the live picture of the service. The inventory is now the
landing page and the first tab, called Home: #home is its address, the older #inventory still resolves to it (every link,
screenshot script and document that names it keeps working), and a bare URL opens there.

Screenshots refreshed so the navigation bar matches; README and the requirements document follow.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/requirements.xlsx
+++ b/docs/requirements.xlsx
@@ -1453,7 +1453,7 @@
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>capacity modelled in Nautobot, enforced by spokes.validate_links, shown on the Inventory page; suites 07 and 10</t>
+          <t>capacity modelled in Nautobot, enforced by spokes.validate_links, shown on the Home page; suites 07 and 10</t>
         </is>
       </c>
     </row>
@@ -2728,7 +2728,7 @@
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>The Inventory page shows the mesh green / red with a live mode (one probe per pair every 5 s, round-trip time in the cell) and columns for the router itself and the internet.</t>
+          <t>The Home page shows the mesh green / red with a live mode (one probe per pair every 5 s, round-trip time in the cell) and columns for the router itself and the internet.</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
@@ -3656,7 +3656,7 @@
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>Inventory: KPIs (Nautobot's VPN model joined with live IKEv2 / VTI / eBGP / ESP state from the headends), a rendered topology (headends on top, spokes below, one line per tunnel coloured by health, hover for details, click to open in Nautobot) and a map of the sites, headend capacity (tunnels, bandwidth, CPU / QFP / DRAM, the binding constraint), the per-tunnel report with CSV export, the LAN hosts and their ping mesh.</t>
+          <t>Home (the landing page; #home, and the older #inventory still resolves): KPIs (Nautobot's VPN model joined with live IKEv2 / VTI / eBGP / ESP state from the headends), a rendered topology (headends on top, spokes below, one line per tunnel coloured by health, hover for details, click to open in Nautobot) and a map of the sites, headend capacity (tunnels, bandwidth, CPU / QFP / DRAM, the binding constraint), the per-tunnel report with CSV export, the LAN hosts and their ping mesh.</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Requirements: the header claimed 60 tests in 11 suites; the delivered system has 74 in 12
The specification's body had kept up with the work (the DCI chain, the Jobs page, Home / Inventory, the queue guard,
the interconnect metrics) but its version block still described the system as it stood on 2026-09-22. Version 1.1 now
states what the last full run measured — 74 tests in 12 suites, 68 passed, 0 failed, 6 skipped, with the skips named —
and TST-01 agrees with it. requirements.pdf and requirements.xlsx rebuilt from the same source (115 requirements in
20 areas, 17 traceability rows, 11 constraints).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/requirements.xlsx
+++ b/docs/requirements.xlsx
@@ -534,7 +534,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>1.0 — 2026-09-22 — derived from the delivered system: every requirement below is implemented and, where stated, verified by the Robot Framework suites (60 tests in 11 suites)</t>
+          <t>1.1 — 2026-09-25 — derived from the delivered system: every requirement below is implemented and, where stated, verified by the Robot Framework suites (74 tests in 12 suites; last full run 68 passed, 0 failed, 6 skipped — the skips are the certificate-mode and portal cases that need a specific starting state)</t>
         </is>
       </c>
     </row>
@@ -4392,7 +4392,7 @@
       </c>
       <c r="E100" s="9" t="inlineStr">
         <is>
-          <t>The whole service is proven by tests against the live lab: 01 management, 02 underlay, 03 IPsec VTI, 04 routing, 05 NaC compliance, 06 Nautobot model, 07 firewalls, 08 PKI, 09 hosts, 10 portal, 11 internet, 12 the DCI chain (incl. the twice-NAT, the DNS fix-up at scale and the packet capture that proves it) — 75 tests; every test reads the expected values from the intent / Nautobot, never from constants.</t>
+          <t>The whole service is proven by tests against the live lab: 01 management, 02 underlay, 03 IPsec VTI, 04 routing, 05 NaC compliance, 06 Nautobot model, 07 firewalls, 08 PKI, 09 hosts, 10 portal, 11 internet, 12 the DCI chain (incl. the twice-NAT, the DNS fix-up at scale and the packet capture that proves it) — 74 tests; every test reads the expected values from the intent / Nautobot, never from constants.</t>
         </is>
       </c>
       <c r="F100" s="9" t="inlineStr">

</xml_diff>